<commit_message>
Label broadcast TYPE ranges with site names in gear table and ops checklist xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014tfFDVXTCXViwumdp6iX1m
</commit_message>
<xml_diff>
--- a/public/dl/STEPIN_Tournament_Ops_Templates.xlsx
+++ b/public/dl/STEPIN_Tournament_Ops_Templates.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
     </font>
     <font>
       <name val="Malgun Gothic"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -84,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -93,6 +97,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -467,7 +474,7 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,6 +484,13 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>중계 형태 (웹사이트 ‘방송 · 중계 셋팅 가이드’와 동일): TYPE 1 체험존 · 현장 랭킹전(중계 없음)  |  TYPE 2 현장 중계(관중용 대형 화면)  |  TYPE 3 녹화 · 현장 스케치  |  TYPE 4 라이브 송출(스트리밍 · 방송사)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -505,7 +519,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>필요 형태</t>
+          <t>필요 중계 형태</t>
         </is>
       </c>
     </row>
@@ -531,7 +545,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>TYPE 1~4</t>
+          <t>전체 형태 (TYPE 1~4)</t>
         </is>
       </c>
     </row>
@@ -557,7 +571,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -583,7 +597,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -609,7 +623,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>TYPE 4</t>
+          <t>라이브 송출 (TYPE 4)</t>
         </is>
       </c>
     </row>
@@ -635,7 +649,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -661,7 +675,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -687,7 +701,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>TYPE 3~4</t>
+          <t>녹화 · 라이브 송출 (TYPE 3~4)</t>
         </is>
       </c>
     </row>
@@ -713,7 +727,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>TYPE 4</t>
+          <t>라이브 송출 (TYPE 4)</t>
         </is>
       </c>
     </row>
@@ -739,7 +753,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -765,7 +779,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -791,7 +805,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -817,7 +831,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>TYPE 1~4</t>
+          <t>전체 형태 (TYPE 1~4)</t>
         </is>
       </c>
     </row>
@@ -843,7 +857,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>TYPE 1~4</t>
+          <t>전체 형태 (TYPE 1~4)</t>
         </is>
       </c>
     </row>
@@ -869,7 +883,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>TYPE 4</t>
+          <t>라이브 송출 (TYPE 4)</t>
         </is>
       </c>
     </row>
@@ -895,7 +909,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -921,7 +935,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -947,7 +961,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -973,7 +987,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -999,7 +1013,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>저조도 · TYPE 2~4</t>
+          <t>저조도 시 · 현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1039,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>TYPE 1~4</t>
+          <t>전체 형태 (TYPE 1~4)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1065,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>TYPE 2~4</t>
+          <t>현장 중계 · 녹화 · 라이브 송출 (TYPE 2~4)</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1091,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>TYPE 1~4</t>
+          <t>전체 형태 (TYPE 1~4)</t>
         </is>
       </c>
     </row>
@@ -1103,11 +1117,14 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>TYPE 1~4</t>
+          <t>전체 형태 (TYPE 1~4)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="D4:D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"O,X"</formula1>

</xml_diff>